<commit_message>
Mejora el CRM con dashboard de funnel, columna Next Action y guiones de Player Opportunities/Development
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -8,17 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Segmento A - Clubes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Segmento B - America" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Segmento C - Becas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="LinkedIn - Plan diario" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Oportunidades y notas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Segmento A - Clubes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Segmento B - America" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Segmento C - Becas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="LinkedIn - Plan diario" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Oportunidades y notas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Segmento A - Clubes'!$A$5:$N$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Segmento B - America'!$A$5:$K$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Segmento C - Becas'!$A$5:$J$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Oportunidades y notas'!$A$4:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Segmento A - Clubes'!$A$5:$O$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Segmento B - America'!$A$5:$N$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Segmento C - Becas'!$A$5:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Oportunidades y notas'!$A$4:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,7 +30,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,7 +59,8 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="11"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -73,6 +75,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -80,6 +88,12 @@
       <i val="1"/>
       <color rgb="007F6000"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -126,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,15 +152,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -513,11 +532,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -546,247 +565,329 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Objetivo diario (LinkedIn + outreach)</t>
+          <t>🔴 URGENTE — mirar esto primero</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Métrica</t>
+          <t>Qué</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Meta diaria</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Hecho hoy (rellenar tú)</t>
+          <t>Cuántos ahora (se calcula solo)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Emails de outreach enviados</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" s="7" t="n"/>
+          <t>Follow-ups de clubes atrasados (enviado hace más de 10 días, sin respuesta)</t>
+        </is>
+      </c>
+      <c r="B6" s="6">
+        <f>COUNTIFS('Segmento A - Clubes'!I2:I300,"Enviado",'Segmento A - Clubes'!M2:M300,"&lt;&gt;",'Segmento A - Clubes'!M2:M300,"&lt;"&amp;(TODAY()-10))+COUNTIFS('Segmento B - America'!H2:H300,"Enviado",'Segmento B - America'!L2:L300,"&lt;&gt;",'Segmento B - America'!L2:L300,"&lt;"&amp;(TODAY()-10))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Búsquedas nuevas de clubes/academias cualificados</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" s="7" t="n"/>
+          <t>Leads de becas con llamada agendada (confirmar/preparar)</t>
+        </is>
+      </c>
+      <c r="B7" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Llamada agendada")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Conexiones de LinkedIn con mensaje personalizado</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
+          <t>Leads de becas cualificados sin próxima acción clara desde hace tiempo (revisar a mano)</t>
+        </is>
+      </c>
+      <c r="B8" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Cualificado")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>🟠 OUTBOUND — lo que generas tú hoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Métrica</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Meta diaria</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Hecho hoy (rellenar tú)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Nuevos clubes/academias investigados</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="7" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Resumen por segmento (se actualiza solo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Segmento</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Total en lista</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Listo para enviar</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Enviado</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Respondido</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Llamada agendada</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Cerrado</t>
-        </is>
-      </c>
+      <c r="C12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Segmento A — Clubes juveniles</t>
-        </is>
-      </c>
-      <c r="B13" s="6">
-        <f>COUNTA('Segmento A - Clubes'!A2:A300)</f>
-        <v/>
-      </c>
-      <c r="C13" s="6">
-        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Listo para enviar")</f>
-        <v/>
-      </c>
-      <c r="D13" s="6">
-        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Enviado")</f>
-        <v/>
-      </c>
-      <c r="E13" s="6">
-        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Respondido")</f>
-        <v/>
-      </c>
-      <c r="F13" s="6">
-        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Llamada agendada")</f>
-        <v/>
-      </c>
-      <c r="G13" s="6">
-        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Cerrado")</f>
-        <v/>
-      </c>
+          <t>Emails de outreach enviados</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Segmento B — Univ./clubes América</t>
-        </is>
-      </c>
-      <c r="B14" s="6">
-        <f>COUNTA('Segmento B - America'!A2:A300)</f>
-        <v/>
-      </c>
-      <c r="C14" s="6">
-        <f>COUNTIF('Segmento B - America'!H2:H300,"Listo para enviar")</f>
-        <v/>
-      </c>
-      <c r="D14" s="6">
-        <f>COUNTIF('Segmento B - America'!H2:H300,"Enviado")</f>
-        <v/>
-      </c>
-      <c r="E14" s="6">
-        <f>COUNTIF('Segmento B - America'!H2:H300,"Respondido")</f>
-        <v/>
-      </c>
-      <c r="F14" s="6">
-        <f>COUNTIF('Segmento B - America'!H2:H300,"Llamada agendada")</f>
-        <v/>
-      </c>
-      <c r="G14" s="6">
-        <f>COUNTIF('Segmento B - America'!H2:H300,"Cerrado")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Segmento C — Becas</t>
-        </is>
-      </c>
+          <t>Conexiones de LinkedIn con mensaje personalizado</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Etapa</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Total</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>🟢 INBOUND — lo que te llega a ti</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="B18" s="6">
-        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Nuevo")</f>
-        <v/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Qué</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Cuántos ahora (se calcula solo)</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Cualificado</t>
+          <t>Leads de becas nuevos sin cualificar todavía</t>
         </is>
       </c>
       <c r="B19" s="6">
-        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Cualificado")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Nuevo")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>📊 PIPELINE — resumen por segmento (detalle completo en pestaña Dashboard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Segmento</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Total en lista</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Listo para enviar</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Respondido</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Llamada agendada</t>
         </is>
       </c>
-      <c r="B20" s="6">
-        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Llamada agendada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Llamada realizada</t>
-        </is>
-      </c>
-      <c r="B21" s="6">
-        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Llamada realizada")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Cerrado</t>
         </is>
-      </c>
-      <c r="B22" s="6">
-        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Cerrado")</f>
-        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
+          <t>Segmento A — Clubes juveniles</t>
+        </is>
+      </c>
+      <c r="B23" s="6">
+        <f>COUNTA('Segmento A - Clubes'!A2:A300)</f>
+        <v/>
+      </c>
+      <c r="C23" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Listo para enviar")</f>
+        <v/>
+      </c>
+      <c r="D23" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Enviado")</f>
+        <v/>
+      </c>
+      <c r="E23" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Respondido")</f>
+        <v/>
+      </c>
+      <c r="F23" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Llamada agendada")</f>
+        <v/>
+      </c>
+      <c r="G23" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Cerrado")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Segmento B — Univ./clubes América</t>
+        </is>
+      </c>
+      <c r="B24" s="6">
+        <f>COUNTA('Segmento B - America'!A2:A300)</f>
+        <v/>
+      </c>
+      <c r="C24" s="6">
+        <f>COUNTIF('Segmento B - America'!H2:H300,"Listo para enviar")</f>
+        <v/>
+      </c>
+      <c r="D24" s="6">
+        <f>COUNTIF('Segmento B - America'!H2:H300,"Enviado")</f>
+        <v/>
+      </c>
+      <c r="E24" s="6">
+        <f>COUNTIF('Segmento B - America'!H2:H300,"Respondido")</f>
+        <v/>
+      </c>
+      <c r="F24" s="6">
+        <f>COUNTIF('Segmento B - America'!H2:H300,"Llamada agendada")</f>
+        <v/>
+      </c>
+      <c r="G24" s="6">
+        <f>COUNTIF('Segmento B - America'!H2:H300,"Cerrado")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Segmento C — Becas</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Etapa</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="B28" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Nuevo")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Cualificado</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Cualificado")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Llamada agendada</t>
+        </is>
+      </c>
+      <c r="B30" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Llamada agendada")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Llamada realizada</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Llamada realizada")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="B32" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Cerrado")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
           <t>Perdido</t>
         </is>
       </c>
-      <c r="B23" s="6">
+      <c r="B33" s="6">
         <f>COUNTIF('Segmento C - Becas'!E2:E300,"Perdido")</f>
         <v/>
       </c>
@@ -806,7 +907,236 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard — funnel por línea de negocio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Estado actual de cada línea. Actualizar Estado/Etapa en las pestañas de segmento — esto se recalcula solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Esto es una FOTO del estado ACTUAL de cada lead (cuántos están ahora mismo en cada estado), no un histórico acumulado de conversión — para eso haría falta guardar fecha de cada cambio de estado, cosa que no hacemos todavía. Sirve igual para ver dónde se acumulan los leads y detectar el cuello de botella real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>TEAM EXPERIENCE  (Segmento A + Segmento B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente investigar</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Listo para enviar</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Respondido</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Llamada agendada</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Llamada realizada</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Pendiente investigar")+COUNTIF('Segmento B - America'!H2:H300,"Pendiente investigar")</f>
+        <v/>
+      </c>
+      <c r="B8" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Listo para enviar")+COUNTIF('Segmento B - America'!H2:H300,"Listo para enviar")</f>
+        <v/>
+      </c>
+      <c r="C8" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Enviado")+COUNTIF('Segmento B - America'!H2:H300,"Enviado")</f>
+        <v/>
+      </c>
+      <c r="D8" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Respondido")+COUNTIF('Segmento B - America'!H2:H300,"Respondido")</f>
+        <v/>
+      </c>
+      <c r="E8" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Llamada agendada")+COUNTIF('Segmento B - America'!H2:H300,"Llamada agendada")</f>
+        <v/>
+      </c>
+      <c r="F8" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Llamada realizada")+COUNTIF('Segmento B - America'!H2:H300,"Llamada realizada")</f>
+        <v/>
+      </c>
+      <c r="G8" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Cerrado")+COUNTIF('Segmento B - America'!H2:H300,"Cerrado")</f>
+        <v/>
+      </c>
+      <c r="H8" s="6">
+        <f>COUNTIF('Segmento A - Clubes'!I2:I300,"Perdido")+COUNTIF('Segmento B - America'!H2:H300,"Perdido")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>BECAS  (Segmento C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Cualificado</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Llamada agendada</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Llamada realizada</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Perdido</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Nuevo")</f>
+        <v/>
+      </c>
+      <c r="B12" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Cualificado")</f>
+        <v/>
+      </c>
+      <c r="C12" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Llamada agendada")</f>
+        <v/>
+      </c>
+      <c r="D12" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Llamada realizada")</f>
+        <v/>
+      </c>
+      <c r="E12" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Cerrado")</f>
+        <v/>
+      </c>
+      <c r="F12" s="6">
+        <f>COUNTIF('Segmento C - Becas'!E2:E300,"Perdido")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>INTERNATIONAL PROGRAM (Real Sociedad)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>0 leads activos todavía — esta sección se activa con el primer lead real. Ver lineas-de-negocio.md línea 3. No crear pestaña de seguimiento hasta entonces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>PLAYER OPPORTUNITIES (Alemania/España) Y PLAYER DEVELOPMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Sin funnel activo — decisión explícita de Joel de no priorizar hasta tener un cliente/jugador real interesado (lineas-de-negocio.md líneas 4 y 6). Si preguntan, ver manual-embudo-ventas.md para el guion de respuesta correcto (nunca prometer prueba/contrato garantizado).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A3:H4"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -818,11 +1148,12 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -840,7 +1171,7 @@
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Prioridad principal (ver plan-ventas-maestro.md sección 3). Estado: usar exactamente estos valores para que las fórmulas de la pestaña Hoy funcionen — Pendiente investigar / Listo para enviar / Enviado / Respondido / Llamada agendada / Llamada realizada / Cerrado / Perdido / En negociación / Solo info.</t>
         </is>
@@ -895,25 +1226,30 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
+          <t>Próxima acción</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
           <t>Asunto email</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>Cuerpo email</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Fecha envío</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Fecha último contacto</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -935,7 +1271,7 @@
           <t>U13-U15 chicas</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Mismo perfil exacto que Greystones (irlandés, viaja a España)</t>
         </is>
@@ -945,7 +1281,7 @@
           <t>dbsportstours.com</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Karl Higgins (U13) / Mark Kelly (U14) / Aaron Doherty (U15)</t>
         </is>
@@ -965,12 +1301,17 @@
           <t>Listo para enviar</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Enviar el email de la columna siguiente hoy</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
         <is>
           <t>Bringing Home Farm FC to train with Atlético de Madrid &amp; Real Sociedad in Spain</t>
         </is>
       </c>
-      <c r="K6" s="10" t="inlineStr">
+      <c r="L6" s="12" t="inlineStr">
         <is>
           <t>Hi Karl / Mark / Aaron,
 I'm Joel, I run Always Up — we bring international youth clubs to Spain to train directly at the facilities of Atletico de Madrid, Real Sociedad and Sporting de Gijon.
@@ -982,9 +1323,9 @@
 Joel</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr"/>
-      <c r="M6" s="6" t="inlineStr"/>
-      <c r="N6" s="10" t="inlineStr">
+      <c r="M6" s="13" t="inlineStr"/>
+      <c r="N6" s="13" t="inlineStr"/>
+      <c r="O6" s="12" t="inlineStr">
         <is>
           <t>Email ya preparado y revisado 2026-08-29 — solo falta que Joel lo envíe</t>
         </is>
@@ -1006,7 +1347,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1016,7 +1357,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Comité juvenil del club</t>
         </is>
@@ -1032,12 +1373,17 @@
           <t>Listo para enviar</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Enviar el email de la columna siguiente esta semana</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
         <is>
           <t>Bringing Søreide IL to train with LaLiga clubs in Spain</t>
         </is>
       </c>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="L7" s="12" t="inlineStr">
         <is>
           <t>Hi,
 I'm Joel, I run Always Up — we bring international youth clubs to Spain to train directly at the facilities of Atletico de Madrid, Real Sociedad and Sporting de Gijon.
@@ -1048,9 +1394,9 @@
 Joel</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="10" t="inlineStr">
+      <c r="M7" s="13" t="inlineStr"/>
+      <c r="N7" s="13" t="inlineStr"/>
+      <c r="O7" s="12" t="inlineStr">
         <is>
           <t>También: fotball@soreideil.no (contacto general del club)</t>
         </is>
@@ -1072,7 +1418,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1082,7 +1428,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>Sin nombre confirmado</t>
         </is>
@@ -1102,11 +1448,16 @@
           <t>Pendiente investigar email</t>
         </is>
       </c>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr"/>
-      <c r="L8" s="6" t="inlineStr"/>
-      <c r="M8" s="6" t="inlineStr"/>
-      <c r="N8" s="10" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Llamar o buscar contacto vía redes del club</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr"/>
+      <c r="L8" s="12" t="inlineStr"/>
+      <c r="M8" s="13" t="inlineStr"/>
+      <c r="N8" s="13" t="inlineStr"/>
+      <c r="O8" s="12" t="inlineStr">
         <is>
           <t>Llamar o contactar vía redes sociales del club para conseguir email directo</t>
         </is>
@@ -1128,7 +1479,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1138,7 +1489,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr"/>
+      <c r="F9" s="12" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr">
@@ -1146,11 +1497,16 @@
           <t>Pendiente investigar</t>
         </is>
       </c>
-      <c r="J9" s="10" t="inlineStr"/>
-      <c r="K9" s="10" t="inlineStr"/>
-      <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="10" t="inlineStr"/>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr"/>
+      <c r="L9" s="12" t="inlineStr"/>
+      <c r="M9" s="13" t="inlineStr"/>
+      <c r="N9" s="13" t="inlineStr"/>
+      <c r="O9" s="12" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -1168,7 +1524,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1178,7 +1534,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr"/>
+      <c r="F10" s="12" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr">
@@ -1186,11 +1542,16 @@
           <t>Pendiente investigar</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr"/>
-      <c r="K10" s="10" t="inlineStr"/>
-      <c r="L10" s="6" t="inlineStr"/>
-      <c r="M10" s="6" t="inlineStr"/>
-      <c r="N10" s="10" t="inlineStr"/>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="inlineStr"/>
+      <c r="L10" s="12" t="inlineStr"/>
+      <c r="M10" s="13" t="inlineStr"/>
+      <c r="N10" s="13" t="inlineStr"/>
+      <c r="O10" s="12" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -1208,7 +1569,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1218,7 +1579,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr"/>
+      <c r="F11" s="12" t="inlineStr"/>
       <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="6" t="inlineStr"/>
       <c r="I11" s="6" t="inlineStr">
@@ -1226,11 +1587,16 @@
           <t>Pendiente investigar</t>
         </is>
       </c>
-      <c r="J11" s="10" t="inlineStr"/>
-      <c r="K11" s="10" t="inlineStr"/>
-      <c r="L11" s="6" t="inlineStr"/>
-      <c r="M11" s="6" t="inlineStr"/>
-      <c r="N11" s="10" t="inlineStr"/>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr"/>
+      <c r="L11" s="12" t="inlineStr"/>
+      <c r="M11" s="13" t="inlineStr"/>
+      <c r="N11" s="13" t="inlineStr"/>
+      <c r="O11" s="12" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -1248,7 +1614,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1258,7 +1624,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F12" s="10" t="inlineStr"/>
+      <c r="F12" s="12" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr">
@@ -1266,11 +1632,16 @@
           <t>Pendiente investigar</t>
         </is>
       </c>
-      <c r="J12" s="10" t="inlineStr"/>
-      <c r="K12" s="10" t="inlineStr"/>
-      <c r="L12" s="6" t="inlineStr"/>
-      <c r="M12" s="6" t="inlineStr"/>
-      <c r="N12" s="10" t="inlineStr"/>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr"/>
+      <c r="L12" s="12" t="inlineStr"/>
+      <c r="M12" s="13" t="inlineStr"/>
+      <c r="N12" s="13" t="inlineStr"/>
+      <c r="O12" s="12" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -1288,7 +1659,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1298,7 +1669,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr"/>
+      <c r="F13" s="12" t="inlineStr"/>
       <c r="G13" s="6" t="inlineStr"/>
       <c r="H13" s="6" t="inlineStr"/>
       <c r="I13" s="6" t="inlineStr">
@@ -1306,11 +1677,16 @@
           <t>Pendiente investigar</t>
         </is>
       </c>
-      <c r="J13" s="10" t="inlineStr"/>
-      <c r="K13" s="10" t="inlineStr"/>
-      <c r="L13" s="6" t="inlineStr"/>
-      <c r="M13" s="6" t="inlineStr"/>
-      <c r="N13" s="10" t="inlineStr"/>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="inlineStr"/>
+      <c r="L13" s="12" t="inlineStr"/>
+      <c r="M13" s="13" t="inlineStr"/>
+      <c r="N13" s="13" t="inlineStr"/>
+      <c r="O13" s="12" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -1328,7 +1704,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1338,7 +1714,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr"/>
+      <c r="F14" s="12" t="inlineStr"/>
       <c r="G14" s="6" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr"/>
       <c r="I14" s="6" t="inlineStr">
@@ -1346,11 +1722,16 @@
           <t>Pendiente investigar</t>
         </is>
       </c>
-      <c r="J14" s="10" t="inlineStr"/>
-      <c r="K14" s="10" t="inlineStr"/>
-      <c r="L14" s="6" t="inlineStr"/>
-      <c r="M14" s="6" t="inlineStr"/>
-      <c r="N14" s="10" t="inlineStr"/>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+        </is>
+      </c>
+      <c r="K14" s="12" t="inlineStr"/>
+      <c r="L14" s="12" t="inlineStr"/>
+      <c r="M14" s="13" t="inlineStr"/>
+      <c r="N14" s="13" t="inlineStr"/>
+      <c r="O14" s="12" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -1368,7 +1749,7 @@
           <t>Sin confirmar</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026</t>
         </is>
@@ -1378,7 +1759,7 @@
           <t>costadauradacup.com</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr"/>
+      <c r="F15" s="12" t="inlineStr"/>
       <c r="G15" s="6" t="inlineStr"/>
       <c r="H15" s="6" t="inlineStr"/>
       <c r="I15" s="6" t="inlineStr">
@@ -1386,11 +1767,16 @@
           <t>Pendiente investigar</t>
         </is>
       </c>
-      <c r="J15" s="10" t="inlineStr"/>
-      <c r="K15" s="10" t="inlineStr"/>
-      <c r="L15" s="6" t="inlineStr"/>
-      <c r="M15" s="6" t="inlineStr"/>
-      <c r="N15" s="10" t="inlineStr"/>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+        </is>
+      </c>
+      <c r="K15" s="12" t="inlineStr"/>
+      <c r="L15" s="12" t="inlineStr"/>
+      <c r="M15" s="13" t="inlineStr"/>
+      <c r="N15" s="13" t="inlineStr"/>
+      <c r="O15" s="12" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -1408,7 +1794,7 @@
           <t>Anfitrión, no viajero</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Posible nuevo club anfitrión — ya en conversación</t>
         </is>
@@ -1418,7 +1804,7 @@
           <t>CLAUDE.md / Joel</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr"/>
+      <c r="F16" s="12" t="inlineStr"/>
       <c r="G16" s="6" t="inlineStr"/>
       <c r="H16" s="6" t="inlineStr"/>
       <c r="I16" s="6" t="inlineStr">
@@ -1426,11 +1812,16 @@
           <t>En negociación</t>
         </is>
       </c>
-      <c r="J16" s="10" t="inlineStr"/>
-      <c r="K16" s="10" t="inlineStr"/>
-      <c r="L16" s="6" t="inlineStr"/>
-      <c r="M16" s="6" t="inlineStr"/>
-      <c r="N16" s="10" t="inlineStr">
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Ver 01-clients/pipeline.md para el estado real</t>
+        </is>
+      </c>
+      <c r="K16" s="12" t="inlineStr"/>
+      <c r="L16" s="12" t="inlineStr"/>
+      <c r="M16" s="13" t="inlineStr"/>
+      <c r="N16" s="13" t="inlineStr"/>
+      <c r="O16" s="12" t="inlineStr">
         <is>
           <t>Ver 01-clients/pipeline.md — no duplicar seguimiento aquí, solo referencia</t>
         </is>
@@ -1452,7 +1843,7 @@
           <t>Sin evaluar</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Contacto personal de Joel, sin explorar todavía</t>
         </is>
@@ -1462,7 +1853,7 @@
           <t>Joel</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr"/>
+      <c r="F17" s="12" t="inlineStr"/>
       <c r="G17" s="6" t="inlineStr"/>
       <c r="H17" s="6" t="inlineStr"/>
       <c r="I17" s="6" t="inlineStr">
@@ -1470,30 +1861,35 @@
           <t>Sin evaluar</t>
         </is>
       </c>
-      <c r="J17" s="10" t="inlineStr"/>
-      <c r="K17" s="10" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="10" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Joel decide si vale la pena explorarlo</t>
+        </is>
+      </c>
+      <c r="K17" s="12" t="inlineStr"/>
+      <c r="L17" s="12" t="inlineStr"/>
+      <c r="M17" s="13" t="inlineStr"/>
+      <c r="N17" s="13" t="inlineStr"/>
+      <c r="O17" s="12" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:N17"/>
+  <autoFilter ref="A5:O17"/>
   <mergeCells count="3">
-    <mergeCell ref="A3:N4"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A3:O4"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1504,9 +1900,12 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1524,7 +1923,7 @@
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>PRIORIDAD SECUNDARIA — ver plan-ventas-maestro.md sección 3. Mercado ya servido por competidores establecidos (Alandis Travel + Sevilla FC, WorldStrides...) y con ciclos de decisión institucionales largos. No forzar volumen aquí hasta tener 2-3 conversaciones reales avanzando en Segmento A.</t>
         </is>
@@ -1574,15 +1973,30 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
+          <t>Próxima acción</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
           <t>Asunto email</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Cuerpo email</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Fecha envío</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>Fecha último contacto</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -1604,7 +2018,7 @@
           <t>Club/Academia</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Participante confirmado Costa Daurada Cup 2026 — encaja con foco geográfico EEUU</t>
         </is>
@@ -1621,9 +2035,16 @@
           <t>Pendiente investigar contacto</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr"/>
-      <c r="J6" s="10" t="inlineStr"/>
-      <c r="K6" s="10" t="inlineStr"/>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>Investigar contacto — solo después de que Segmento A tenga 2-3 conversaciones reales</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr"/>
+      <c r="K6" s="12" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr"/>
+      <c r="M6" s="13" t="inlineStr"/>
+      <c r="N6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -1641,7 +2062,7 @@
           <t>Club/Academia (ECNL)</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Participante ECNL International IberCup 2026</t>
         </is>
@@ -1658,9 +2079,16 @@
           <t>Pendiente filtrar por edad + contacto</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr"/>
-      <c r="J7" s="10" t="inlineStr"/>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar categorías mayores antes de investigar más</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr"/>
+      <c r="K7" s="12" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr"/>
+      <c r="M7" s="13" t="inlineStr"/>
+      <c r="N7" s="12" t="inlineStr">
         <is>
           <t>Aviso: categoría IberCup es U11/U12 7v7 — confirmar que tienen categorías mayores antes de contactar</t>
         </is>
@@ -1682,7 +2110,7 @@
           <t>Club/Academia (ECNL)</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Participante ECNL International IberCup 2026</t>
         </is>
@@ -1699,9 +2127,16 @@
           <t>Pendiente filtrar por edad + contacto</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr"/>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar categorías mayores antes de investigar más</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr"/>
+      <c r="K8" s="12" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr"/>
+      <c r="M8" s="13" t="inlineStr"/>
+      <c r="N8" s="12" t="inlineStr">
         <is>
           <t>Mismo aviso de edad que arriba</t>
         </is>
@@ -1723,7 +2158,7 @@
           <t>Club/Academia (ECNL)</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Participante ECNL International IberCup 2026</t>
         </is>
@@ -1740,9 +2175,16 @@
           <t>Pendiente filtrar por edad + contacto</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr"/>
-      <c r="J9" s="10" t="inlineStr"/>
-      <c r="K9" s="10" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar categorías mayores antes de investigar más</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr"/>
+      <c r="K9" s="12" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr"/>
+      <c r="M9" s="13" t="inlineStr"/>
+      <c r="N9" s="12" t="inlineStr">
         <is>
           <t>Mismo aviso de edad que arriba</t>
         </is>
@@ -1764,7 +2206,7 @@
           <t>Club/Academia (ECNL)</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Participante ECNL International IberCup 2026</t>
         </is>
@@ -1781,9 +2223,16 @@
           <t>Pendiente filtrar por edad + contacto</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr"/>
-      <c r="J10" s="10" t="inlineStr"/>
-      <c r="K10" s="10" t="inlineStr">
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar categorías mayores antes de investigar más</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr"/>
+      <c r="K10" s="12" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr"/>
+      <c r="M10" s="13" t="inlineStr"/>
+      <c r="N10" s="12" t="inlineStr">
         <is>
           <t>Mismo aviso de edad que arriba</t>
         </is>
@@ -1805,7 +2254,7 @@
           <t>Club/Academia (ECNL)</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Participante ECNL International IberCup 2026</t>
         </is>
@@ -1822,9 +2271,16 @@
           <t>Pendiente filtrar por edad + contacto</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr"/>
-      <c r="J11" s="10" t="inlineStr"/>
-      <c r="K11" s="10" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar categorías mayores antes de investigar más</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr"/>
+      <c r="K11" s="12" t="inlineStr"/>
+      <c r="L11" s="13" t="inlineStr"/>
+      <c r="M11" s="13" t="inlineStr"/>
+      <c r="N11" s="12" t="inlineStr">
         <is>
           <t>Mismo aviso de edad que arriba</t>
         </is>
@@ -1846,7 +2302,7 @@
           <t>NCAA D1 (ACC, top-25)</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Primera gira internacional en 15 años (Dublín, agosto 2026) — demuestra que el interés es real</t>
         </is>
@@ -1863,9 +2319,16 @@
           <t>Solo referencia — NO contactar</t>
         </is>
       </c>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="10" t="inlineStr"/>
-      <c r="K12" s="10" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>Ninguna — caso de estudio, no target</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr"/>
+      <c r="K12" s="12" t="inlineStr"/>
+      <c r="L12" s="13" t="inlineStr"/>
+      <c r="M12" s="13" t="inlineStr"/>
+      <c r="N12" s="12" t="inlineStr">
         <is>
           <t>Programa grande con relaciones ya asentadas, mal candidato para primer contacto. Dejar como caso de estudio del mercado</t>
         </is>
@@ -1887,7 +2350,7 @@
           <t>NCAA D2/D3</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Hipótesis sin validar: menos competencia que D1, presupuestos más flexibles</t>
         </is>
@@ -1904,26 +2367,33 @@
           <t>Pendiente investigación profunda</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr"/>
-      <c r="J13" s="10" t="inlineStr"/>
-      <c r="K13" s="10" t="inlineStr">
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Sesión de investigación dedicada (no urgente)</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr"/>
+      <c r="K13" s="12" t="inlineStr"/>
+      <c r="L13" s="13" t="inlineStr"/>
+      <c r="M13" s="13" t="inlineStr"/>
+      <c r="N13" s="12" t="inlineStr">
         <is>
           <t>Búsqueda rápida (2026-08-29) no encontró candidatos concretos — requiere sesión de investigación dedicada, no una búsqueda genérica</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:K13"/>
+  <autoFilter ref="A5:N13"/>
   <mergeCells count="3">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K4"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A3:N4"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1959,7 +2429,7 @@
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>MIGRADO desde 01-clients/pipeline.md (tabla 'Embudo — seguimiento de leads inbound') el 2026-08-29 — esta pestaña sustituye esa tabla como fuente única de verdad para leads de becas. Etapa: usar Nuevo / Cualificado / Llamada agendada / Llamada realizada / Cerrado / Perdido para que las fórmulas de Hoy funcionen.</t>
         </is>
@@ -2054,7 +2524,7 @@
           <t>Sí — mandó vídeo</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>Acusar recibo del vídeo y evaluar</t>
         </is>
@@ -2064,7 +2534,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>Dilema real: ir a EEUU 2027 vs. quedarse en Portugal a estudiar</t>
         </is>
@@ -2094,7 +2564,7 @@
           <t>Sin evaluar</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>Aceptar la solicitud de IG (2 semanas sin aceptar)</t>
         </is>
@@ -2104,7 +2574,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>Preguntó directamente por el sistema de becas</t>
         </is>
@@ -2146,7 +2616,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>Proponer videollamada</t>
         </is>
@@ -2156,7 +2626,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J8" s="10" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>Lead fuerte — ya en EEUU, quiere seguir compitiendo y sacar diploma</t>
         </is>
@@ -2182,7 +2652,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>Confirmar hora propuesta: jueves 8am</t>
         </is>
@@ -2192,7 +2662,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>Lead muy caliente, solo falta confirmar</t>
         </is>
@@ -2218,7 +2688,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>Confirmar día para videollamada</t>
         </is>
@@ -2228,7 +2698,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>Intentaba cerrar día ('hoy o mañana'), se quedó sin respuesta</t>
         </is>
@@ -2270,7 +2740,7 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>Enviar explicación del proceso EEUU (nunca mencionar University Soccer)</t>
         </is>
@@ -2280,7 +2750,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J11" s="10" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>Originalmente pedía Inglaterra, aceptó explorar vía EEUU</t>
         </is>
@@ -2322,7 +2792,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>Pedir el vídeo (de mayo 2026, ya lo tienen listo)</t>
         </is>
@@ -2332,7 +2802,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J12" s="10" t="inlineStr">
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>Datos completos, solo falta el vídeo</t>
         </is>
@@ -2370,7 +2840,7 @@
           <t>Parcial — edad muy temprana para evaluar</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
         <is>
           <t>Enviar guia-becas.md</t>
         </is>
@@ -2380,7 +2850,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J13" s="10" t="inlineStr">
+      <c r="J13" s="12" t="inlineStr">
         <is>
           <t>Pidió la guía explícitamente</t>
         </is>
@@ -2414,7 +2884,7 @@
           <t>Sí, pero enfriado</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>Reactivar — el enlace genérico anterior no tuvo CTA claro</t>
         </is>
@@ -2424,7 +2894,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J14" s="10" t="inlineStr">
+      <c r="J14" s="12" t="inlineStr">
         <is>
           <t>Conversación avanzada que se enfrió</t>
         </is>
@@ -2466,7 +2936,7 @@
           <t>Parcial — edad temprana</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>Seguir conversación</t>
         </is>
@@ -2476,7 +2946,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J15" s="10" t="inlineStr"/>
+      <c r="J15" s="12" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -2510,7 +2980,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>Responder pregunta directa sobre inscripción</t>
         </is>
@@ -2520,7 +2990,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J16" s="10" t="inlineStr"/>
+      <c r="J16" s="12" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -2554,7 +3024,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H17" s="12" t="inlineStr">
         <is>
           <t>Pedir vídeo y notas académicas</t>
         </is>
@@ -2564,7 +3034,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J17" s="10" t="inlineStr">
+      <c r="J17" s="12" t="inlineStr">
         <is>
           <t>Confirmado: Always Up sí trabaja otros deportes, no solo fútbol</t>
         </is>
@@ -2606,7 +3076,7 @@
           <t>Parcial — falta situación académica</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H18" s="12" t="inlineStr">
         <is>
           <t>Pedir situación académica</t>
         </is>
@@ -2616,7 +3086,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J18" s="10" t="inlineStr">
+      <c r="J18" s="12" t="inlineStr">
         <is>
           <t>Cuenta confirmada por Joel — verificar en próximo barrido</t>
         </is>
@@ -2646,7 +3116,7 @@
           <t>No — respuesta muy breve</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="H19" s="12" t="inlineStr">
         <is>
           <t>Verificar que el mensaje le llegó bien (aviso de cuenta restringida)</t>
         </is>
@@ -2656,7 +3126,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J19" s="10" t="inlineStr"/>
+      <c r="J19" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:J19"/>
@@ -2669,7 +3139,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2701,7 +3171,7 @@
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Pestaña plantilla — se activa cuando el perfil de LinkedIn esté pulido (roadmap-maestro.md tarea #8, sesión conjunta pendiente con Claude in Chrome). Reglas de mensaje: ver plan-ventas-maestro.md sección 4 — siempre a una persona con cargo concreto, con una señal real (post/torneo/resultado), nunca plantilla fría.</t>
         </is>
@@ -2746,7 +3216,7 @@
       <c r="C6" s="6" t="inlineStr"/>
       <c r="D6" s="6" t="inlineStr"/>
       <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="10" t="inlineStr"/>
+      <c r="F6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr"/>
@@ -2754,7 +3224,7 @@
       <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="10" t="inlineStr"/>
+      <c r="F7" s="12" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr"/>
@@ -2762,7 +3232,7 @@
       <c r="C8" s="6" t="inlineStr"/>
       <c r="D8" s="6" t="inlineStr"/>
       <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="10" t="inlineStr"/>
+      <c r="F8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr"/>
@@ -2770,7 +3240,7 @@
       <c r="C9" s="6" t="inlineStr"/>
       <c r="D9" s="6" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="10" t="inlineStr"/>
+      <c r="F9" s="12" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr"/>
@@ -2778,7 +3248,7 @@
       <c r="C10" s="6" t="inlineStr"/>
       <c r="D10" s="6" t="inlineStr"/>
       <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="10" t="inlineStr"/>
+      <c r="F10" s="12" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr"/>
@@ -2786,7 +3256,7 @@
       <c r="C11" s="6" t="inlineStr"/>
       <c r="D11" s="6" t="inlineStr"/>
       <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="10" t="inlineStr"/>
+      <c r="F11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr"/>
@@ -2794,7 +3264,7 @@
       <c r="C12" s="6" t="inlineStr"/>
       <c r="D12" s="6" t="inlineStr"/>
       <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="10" t="inlineStr"/>
+      <c r="F12" s="12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2830,7 +3300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2862,7 +3332,7 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Backlog ligero para líneas que aún no tienen operativa propia de venta — no crear pestañas dedicadas hasta que Joel las eleve de prioridad (ver roadmap-maestro.md).</t>
         </is>
@@ -2911,7 +3381,7 @@
           <t>International Program (Real Sociedad)</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Cerrar % de comisión con la Real Sociedad</t>
         </is>
@@ -2921,7 +3391,7 @@
           <t>roadmap-maestro.md #6</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Bajado de prioridad — no mueve el cuello de botella actual</t>
         </is>
@@ -2943,7 +3413,7 @@
           <t>Puerto Rico / SADE Soccer Academy</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Showcase conectado a la Real Sociedad, facilitado por David</t>
         </is>
@@ -2953,7 +3423,7 @@
           <t>lineas-de-negocio.md</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Confirmado que pasa por Always Up — seguir según avance David</t>
         </is>
@@ -2975,7 +3445,7 @@
           <t>Alemania/España</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Oportunidades profesionales — objetivo 2027</t>
         </is>
@@ -2985,7 +3455,7 @@
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Sin estructurar todavía, no es foco actual</t>
         </is>
@@ -3007,7 +3477,7 @@
           <t>Always Up Player Development</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Academia de formación de jugadores (línea 6)</t>
         </is>
@@ -3017,7 +3487,7 @@
           <t>lineas-de-negocio.md</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Ritmo propio, ligado a marca personal — sesión aparte</t>
         </is>
@@ -3039,7 +3509,7 @@
           <t>Segmento B (NCAA)</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Programas NCAA D2/D3 sin partnership de tours visible</t>
         </is>
@@ -3049,7 +3519,7 @@
           <t>plan-ventas-maestro.md</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Requiere sesión de investigación dedicada — búsqueda rápida no encontró candidatos concretos</t>
         </is>

</xml_diff>

<commit_message>
Investiga 4 clubes nuevos de Segmento A (Hastings United listo para enviar)
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -1466,7 +1466,7 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Whitehaven AFC</t>
+          <t>Whitehaven AFC (Juniors Girls U13-U15)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1476,37 +1476,49 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Sin confirmar</t>
+          <t>U13-U15 chicas</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Participante confirmado Costa Daurada Cup 2026</t>
+          <t>Participante confirmado Costa Daurada Cup 2026 + tiene estructura de chicas U13/U14/U15 activa (The FA Full-Time)</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>costadauradacup.com</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
+          <t>costadauradacup.com / fulltime.thefa.com</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Sin nombre confirmado todavía</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Sin email directo — solo formulario en whitehavenafc.com/contact</t>
+        </is>
+      </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar</t>
+          <t>Pendiente investigar decisor</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+          <t>Rellenar el formulario de contacto o buscar el nombre del responsable de chicas en redes del club antes de escribir</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr"/>
       <c r="L9" s="12" t="inlineStr"/>
       <c r="M9" s="13" t="inlineStr"/>
       <c r="N9" s="13" t="inlineStr"/>
-      <c r="O9" s="12" t="inlineStr"/>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>Investigado 2026-08-29: club real con categorías U13-U15 chicas, pero sin decisor nombrado todavía — no está al nivel de Home Farm/Hastings todavía</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -1516,7 +1528,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Reino Unido (sin confirmar)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1526,7 +1538,7 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Participante confirmado Costa Daurada Cup 2026</t>
+          <t>Aparecía como participante Costa Daurada Cup 2026 en el research original de julio</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1539,19 +1551,23 @@
       <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar</t>
+          <t>Sin identificar con certeza</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+          <t>Verificar directamente en costadauradacup.com — la búsqueda de hoy solo encontró clubes de Ormond en Australia (deporte distinto, AFL), no coincide</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr"/>
       <c r="L10" s="12" t="inlineStr"/>
       <c r="M10" s="13" t="inlineStr"/>
       <c r="N10" s="13" t="inlineStr"/>
-      <c r="O10" s="12" t="inlineStr"/>
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -1566,42 +1582,58 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Sin confirmar</t>
+          <t>Estructura U7-U14+</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Participante confirmado Costa Daurada Cup 2026</t>
+          <t>Participante confirmado Costa Daurada Cup 2026 + club con estructura juvenil real y activa</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>costadauradacup.com</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="6" t="inlineStr"/>
+          <t>costadauradacup.com / holbeachunitedcsa.org.uk</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Sin nombre confirmado todavía</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>info@holbeachunitedcsa.org.uk</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>07801 049254</t>
+        </is>
+      </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar</t>
+          <t>Pendiente investigar decisor</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+          <t>Escribir al email general pidiendo hablar con el responsable de viajes/categorías mayores antes de mandar la propuesta completa</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr"/>
       <c r="L11" s="12" t="inlineStr"/>
       <c r="M11" s="13" t="inlineStr"/>
       <c r="N11" s="13" t="inlineStr"/>
-      <c r="O11" s="12" t="inlineStr"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>Investigado 2026-08-29: contacto general real, falta nombre de decisor</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Hastings United</t>
+          <t>Hastings United (Girls Academy)</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1611,37 +1643,63 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Sin confirmar</t>
+          <t>Academia — chicas</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Participante confirmado Costa Daurada Cup 2026</t>
+          <t>Participante confirmado Costa Daurada Cup 2026 + academia estructurada con Head of Girls Academy identificada</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>costadauradacup.com</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
+          <t>costadauradacup.com / academy.hastingsunited.com</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Georgia Townsend (Head of Girls Academy)</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>georgia.townsend@hastingsunited.com</t>
+        </is>
+      </c>
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar</t>
+          <t>Listo para enviar</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
-        </is>
-      </c>
-      <c r="K12" s="12" t="inlineStr"/>
-      <c r="L12" s="12" t="inlineStr"/>
+          <t>Enviar el email de la columna siguiente esta semana</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>Bringing Hastings United's Girls Academy to train with LaLiga clubs in Spain</t>
+        </is>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>Hi Georgia,
+I'm Joel, founder of Always Up — we create football experiences in Spain for international youth clubs, including training connected with Atletico de Madrid and Real Sociedad.
+I saw Hastings United is a confirmed participant in the Costa Daurada Cup 2026 and thought this could be a great fit for your Girls Academy.
+One of our longtime partner clubs credited their first-ever league title partly to their Atletico de Madrid experience with us — and with Spain now World Cup Champions, interest in trips like this is only growing.
+Would you have 15 minutes this week to hear more?
+Best,
+Joel</t>
+        </is>
+      </c>
       <c r="M12" s="13" t="inlineStr"/>
       <c r="N12" s="13" t="inlineStr"/>
-      <c r="O12" s="12" t="inlineStr"/>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>Investigado 2026-08-29: el mejor de los 4 investigados hoy — decisor nombrado y academia real</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -1651,7 +1709,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Reino Unido (verificar)</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1661,7 +1719,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Participante confirmado Costa Daurada Cup 2026</t>
+          <t>Aparecía como participante Costa Daurada Cup 2026 en el research original de julio</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1670,23 +1728,31 @@
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr"/>
-      <c r="G13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>office@morecambefc.com (club matriz, sin confirmar relación)</t>
+        </is>
+      </c>
       <c r="H13" s="6" t="inlineStr"/>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar</t>
+          <t>Verificar antes de contactar</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
+          <t>La búsqueda de hoy solo encontró 'Morecambe Hawks United MHU', equipo de liga local pequeña — verificar si es el mismo club antes de escribir, puede ser coincidencia de nombre</t>
         </is>
       </c>
       <c r="K13" s="12" t="inlineStr"/>
       <c r="L13" s="12" t="inlineStr"/>
       <c r="M13" s="13" t="inlineStr"/>
       <c r="N13" s="13" t="inlineStr"/>
-      <c r="O13" s="12" t="inlineStr"/>
+      <c r="O13" s="12" t="inlineStr">
+        <is>
+          <t>Investigado 2026-08-29: discrepancia entre el research original y lo encontrado hoy — no mandar nada hasta confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="6" t="inlineStr">

</xml_diff>